<commit_message>
Balancing-Liste: Koedersender behaelt Aggro, nur Taunt gestrichen
Auf Rueckmeldung: EQP-008 bleibt als Gadget mit seiner normalen Aggro (+25)
drin; nur die Provokation/der Taunt (Stoersignal) faellt weg.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D3vVboPsRiuUSAKfufCxCH
</commit_message>
<xml_diff>
--- a/docs/ausruestung_stats.xlsx
+++ b/docs/ausruestung_stats.xlsx
@@ -17,7 +17,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Huelle'!$A$4:$M$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Waffen'!$A$4:$J$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Kerne'!$A$4:$K$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Gadgets'!$A$4:$F$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Gadgets'!$A$4:$F$8</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -502,7 +502,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C60"/>
+  <dimension ref="A1:C61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1004,66 +1004,73 @@
     <row r="51">
       <c r="A51" s="7" t="inlineStr">
         <is>
-          <t>Der Koedersender (EQP-008) ist auf Wunsch vorerst gestrichen.</t>
+          <t>Der Koedersender (EQP-008) behaelt seine normale Aggro (+25) -- nur der</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="7" t="inlineStr"/>
+      <c r="A52" s="7" t="inlineStr">
+        <is>
+          <t>Taunt/die Provokation (Stoersignal) ist gestrichen.</t>
+        </is>
+      </c>
     </row>
     <row r="53">
-      <c r="A53" s="7" t="inlineStr">
-        <is>
-          <t>Schema: je Kategorie eine Liste 'spalten' (key, label, kind, width) und eine</t>
-        </is>
-      </c>
+      <c r="A53" s="7" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="7" t="inlineStr">
         <is>
-          <t>Liste 'zeilen'. kind='stat' sind die getunten Zahlen (in der Mappe</t>
+          <t>Schema: je Kategorie eine Liste 'spalten' (key, label, kind, width) und eine</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="7" t="inlineStr">
         <is>
+          <t>Liste 'zeilen'. kind='stat' sind die getunten Zahlen (in der Mappe</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="7" t="inlineStr">
+        <is>
           <t>hervorgehoben), 'desc' beschreibender Text, 'id'/'text' der Rest. Neue Spalte</t>
         </is>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" s="7">
+    <row r="57">
+      <c r="A57" s="7">
         <f> ein Eintrag in 'spalten' plus das Feld in jeder Zeile.</f>
         <v/>
       </c>
     </row>
-    <row r="57">
-      <c r="A57" s="7" t="inlineStr"/>
-    </row>
     <row r="58">
-      <c r="A58" s="7" t="inlineStr">
-        <is>
-          <t>Arbeitsweise: Werte hier (oder in der Excel-Mappe) aendern, dann</t>
-        </is>
-      </c>
+      <c r="A58" s="7" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">  python3 tools/build_balance_sheet.py</t>
+          <t>Arbeitsweise: Werte hier (oder in der Excel-Mappe) aendern, dann</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="7" t="inlineStr">
         <is>
+          <t xml:space="preserve">  python3 tools/build_balance_sheet.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="7" t="inlineStr">
+        <is>
           <t>erzeugt docs/ausruestung_stats.xlsx neu.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="33">
+  <mergeCells count="34">
     <mergeCell ref="A41:C41"/>
     <mergeCell ref="A37:C37"/>
     <mergeCell ref="A46:C46"/>
@@ -1096,6 +1103,7 @@
     <mergeCell ref="A36:C36"/>
     <mergeCell ref="A49:C49"/>
     <mergeCell ref="A45:C45"/>
+    <mergeCell ref="A61:C61"/>
     <mergeCell ref="A54:C54"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2077,7 +2085,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2098,7 +2106,7 @@
     <row r="2" ht="28" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Support und Schild. Je Teil ein Wert (je Teil ein anderer) plus Wirkungstext. Koedersender vorerst gestrichen.</t>
+          <t>Support und Schild. Je Teil ein Wert (je Teil ein anderer) plus Wirkungstext. Koedersender: Aggro bleibt, Taunt gestrichen.</t>
         </is>
       </c>
     </row>
@@ -2224,8 +2232,38 @@
         </is>
       </c>
     </row>
+    <row r="8" ht="44" customHeight="1">
+      <c r="A8" s="10" t="inlineStr">
+        <is>
+          <t>EQP-008</t>
+        </is>
+      </c>
+      <c r="B8" s="10" t="inlineStr">
+        <is>
+          <t>Koedersender</t>
+        </is>
+      </c>
+      <c r="C8" s="10" t="inlineStr">
+        <is>
+          <t>Support</t>
+        </is>
+      </c>
+      <c r="D8" s="10" t="inlineStr">
+        <is>
+          <t>Aggro</t>
+        </is>
+      </c>
+      <c r="E8" s="9" t="n">
+        <v>25</v>
+      </c>
+      <c r="F8" s="10" t="inlineStr">
+        <is>
+          <t>Erzeugt zusätzliche Aggro (+25) -- zieht Aufmerksamkeit auf sich. Ohne Taunt/Provokation (Stoersignal gestrichen).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:F7"/>
+  <autoFilter ref="A4:F8"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>